<commit_message>
Actualiza el GDD a la versión 0.3.1 con interfaz y avance del prototipo
</commit_message>
<xml_diff>
--- a/AfterLight_Stats.xlsx
+++ b/AfterLight_Stats.xlsx
@@ -333,7 +333,7 @@
     <t>Óptica de largo alcance</t>
   </si>
   <si>
-    <t>+1 m al alcance de la linterna.</t>
+    <t>+2.4 m al alcance de la linterna.</t>
   </si>
   <si>
     <t>CAR-009</t>
@@ -405,7 +405,7 @@
     <t>Calibración balística</t>
   </si>
   <si>
-    <t>+1 m al alcance efectivo del arma equipada.</t>
+    <t>+2.4 m al alcance efectivo del arma equipada.</t>
   </si>
   <si>
     <t>CAR-017</t>
@@ -414,7 +414,7 @@
     <t>Paso ligero</t>
   </si>
   <si>
-    <t>+0.3 m/s a la velocidad normal.</t>
+    <t>+0.72 m/s a la velocidad normal.</t>
   </si>
   <si>
     <t>CAR-018</t>
@@ -423,7 +423,7 @@
     <t>Avance táctico</t>
   </si>
   <si>
-    <t>+0.25 m/s al apuntar, sin superar velocidad normal.</t>
+    <t>+0.6 m/s al apuntar, sin superar velocidad normal.</t>
   </si>
   <si>
     <t>CAR-019</t>
@@ -441,7 +441,7 @@
     <t>Recolector magnético</t>
   </si>
   <si>
-    <t>+0.5 m al radio de recolección.</t>
+    <t>+1.2 m al radio de recolección.</t>
   </si>
   <si>
     <t>CAR-021</t>
@@ -1093,8 +1093,8 @@
       <c r="B16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="10">
-        <v>8</v>
+      <c r="C16" s="11">
+        <v>19.2</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>36</v>
@@ -1201,8 +1201,8 @@
       <c r="B22" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="7">
-        <v>12</v>
+      <c r="C22" s="8">
+        <v>28.8</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>36</v>
@@ -1256,7 +1256,7 @@
         <v>58</v>
       </c>
       <c r="C25" s="11">
-        <v>4.5</v>
+        <v>10.8</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>59</v>
@@ -1274,7 +1274,7 @@
         <v>61</v>
       </c>
       <c r="C26" s="8">
-        <v>3.5</v>
+        <v>8.4</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>59</v>
@@ -1310,7 +1310,7 @@
         <v>67</v>
       </c>
       <c r="C28" s="8">
-        <v>1.5</v>
+        <v>3.6</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>36</v>

</xml_diff>